<commit_message>
Update Automation Work Plan: promote Governance Monitoring and Stakeholder Communications to Wave 2
Adds Governance Monitoring (1.3) and Stakeholder Communications (1.4) as Wave 2b and 2c workstreams with full deliverable breakdowns (4 deliverables each). Renumbers Personal Task Management to 1.5 (Wave 3a) and Strategic Resourcing to 1.6 (Wave 3b). Updates Gantt chart with new rows for both new workstreams and corrected legend. Updates React frontend screen names to reflect new workstream set.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI PMO Tool - Automation Work Plan.xlsx
+++ b/AI PMO Tool - Automation Work Plan.xlsx
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -180,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -194,11 +194,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -224,7 +252,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -242,7 +270,7 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -260,7 +288,7 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -325,6 +353,18 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -690,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -833,7 +873,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="50" t="n">
         <v>46295</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -860,7 +900,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Build the EPAM-branded React (TypeScript) web application scaffold: routing, authentication flow, component library, responsive layout for desktop and mobile, and the five core screens (Dashboard, Review Queue, Task Checklist, Report Approval, Resource Alerts). Azure AD SSO integration via MSAL so PMOs log in with their existing organisational credentials.</t>
+          <t>Build the EPAM-branded React (TypeScript) web application scaffold: routing, authentication flow, component library, responsive layout for desktop and mobile, and the five core screens (Dashboard, Review Queue, Governance Dashboard, Report Approval, Stakeholder Communications). Azure AD SSO integration via MSAL so PMOs log in with their existing organisational credentials.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -873,7 +913,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="50" t="n">
         <v>46295</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -913,7 +953,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="50" t="n">
         <v>46312</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -953,7 +993,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="50" t="n">
         <v>46312</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1042,7 +1082,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="51" t="n">
         <v>46340</v>
       </c>
       <c r="G16" s="13" t="inlineStr">
@@ -1082,7 +1122,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="51" t="n">
         <v>46340</v>
       </c>
       <c r="G17" s="13" t="inlineStr">
@@ -1122,7 +1162,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="51" t="n">
         <v>46368</v>
       </c>
       <c r="G18" s="13" t="inlineStr">
@@ -1162,7 +1202,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="51" t="n">
         <v>46368</v>
       </c>
       <c r="G19" s="13" t="inlineStr">
@@ -1202,7 +1242,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F20" s="15" t="n">
+      <c r="F20" s="51" t="n">
         <v>46396</v>
       </c>
       <c r="G20" s="13" t="inlineStr">
@@ -1242,7 +1282,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n">
+      <c r="F21" s="51" t="n">
         <v>46396</v>
       </c>
       <c r="G21" s="13" t="inlineStr">
@@ -1282,7 +1322,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F22" s="15" t="n">
+      <c r="F22" s="51" t="n">
         <v>46396</v>
       </c>
       <c r="G22" s="13" t="inlineStr">
@@ -1322,7 +1362,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F23" s="15" t="n">
+      <c r="F23" s="51" t="n">
         <v>46417</v>
       </c>
       <c r="G23" s="13" t="inlineStr">
@@ -1362,7 +1402,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F24" s="15" t="n">
+      <c r="F24" s="51" t="n">
         <v>46417</v>
       </c>
       <c r="G24" s="13" t="inlineStr">
@@ -1451,7 +1491,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F28" s="21" t="n">
+      <c r="F28" s="52" t="n">
         <v>46459</v>
       </c>
       <c r="G28" s="19" t="inlineStr">
@@ -1491,7 +1531,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F29" s="21" t="n">
+      <c r="F29" s="52" t="n">
         <v>46459</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
@@ -1531,7 +1571,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F30" s="21" t="n">
+      <c r="F30" s="52" t="n">
         <v>46488</v>
       </c>
       <c r="G30" s="19" t="inlineStr">
@@ -1571,7 +1611,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F31" s="21" t="n">
+      <c r="F31" s="52" t="n">
         <v>46488</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
@@ -1611,7 +1651,7 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F32" s="21" t="n">
+      <c r="F32" s="52" t="n">
         <v>46516</v>
       </c>
       <c r="G32" s="19" t="inlineStr">
@@ -1625,74 +1665,114 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>1.3  Wave 2b - Governance Monitoring</t>
+        </is>
+      </c>
+    </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>1.3  Wave 2b - Personal Task Management</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Deliverable Name</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Deliverable Description</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Project Description</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Delivery Owner</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Document Name</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Technological Uncertainties</t>
         </is>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Deliverable Name</t>
-        </is>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>Deliverable Description</t>
-        </is>
-      </c>
-      <c r="D35" s="17" t="inlineStr">
-        <is>
-          <t>Project Description</t>
-        </is>
-      </c>
-      <c r="E35" s="17" t="inlineStr">
-        <is>
-          <t>Delivery Owner</t>
-        </is>
-      </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="G35" s="17" t="inlineStr">
-        <is>
-          <t>Document Name</t>
-        </is>
-      </c>
-      <c r="H35" s="17" t="inlineStr">
-        <is>
-          <t>Technological Uncertainties</t>
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>Governance Standards Configuration &amp; Assessment Engine</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Build the configurable governance standards store: per-client rule sets defining what is checked, the evidence source (SharePoint document, RAID log entry, JIRA field), review cadence, and breach severity (High/Medium/Low). Implement the automated assessment engine running weekly scheduled checks and on-demand assessments against all active projects. Standards are versionable with a full change audit log. PMO Lead can configure and update standards without code changes.</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Wave 2 Governance Monitoring delivers continuous automated assessment of every active project against configured governance standards - checking documentation, approvals, and gate criteria. It draws on Wave 1 RAID logs and decision records as primary evidence, generates per-project governance scorecards, detects gaps by type and severity, and surfaces escalation drafts for PMO review. All gap resolutions require explicit PMO action - the system detects and surfaces, humans resolve and dismiss.</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F35" s="52" t="n">
+        <v>46459</v>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>Governance Standards Config Spec &amp; Assessment Engine Design</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>Governance standards vary significantly by client and may require dedicated discovery sessions before configuration can begin.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>1.3.2</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Email Commitment Extraction Agent</t>
+          <t>Gap Detection &amp; Classification Module</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Develop the LLM-based agent that connects to the PMO Outlook inbox via Microsoft Graph API, scans over a configurable lookback window (default 3 days), identifies commitments made by and tasks directed at the PMO, and distinguishes hard commitments from soft commitments and FYI information. Extracted tasks surfaced in the EPAM platform.</t>
+          <t>Build the module evaluating assessment results and classifying each gap by type (Missing Document, Overdue Approval, Overdue Review, Unresolved Change Request, Governance Gate Failure) and severity (High/Medium/Low). Implement duplicate suppression so persistent gaps age in place rather than being re-raised each cycle. High severity gaps trigger immediate PMO notification. Each gap record includes: breached standard, expected evidence, evidence found, first detected date, and duration open.</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+          <t>Wave 2 Governance Monitoring delivers continuous automated assessment of every active project against configured governance standards - checking documentation, approvals, and gate criteria. It draws on Wave 1 RAID logs and decision records as primary evidence, generates per-project governance scorecards, detects gaps by type and severity, and surfaces escalation drafts for PMO review. All gap resolutions require explicit PMO action - the system detects and surfaces, humans resolve and dismiss.</t>
         </is>
       </c>
       <c r="E36" s="20" t="inlineStr">
@@ -1700,39 +1780,39 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F36" s="21" t="n">
-        <v>46459</v>
+      <c r="F36" s="52" t="n">
+        <v>46488</v>
       </c>
       <c r="G36" s="19" t="inlineStr">
         <is>
-          <t>Email Agent - Accuracy Evaluation &amp; PII Handling Report</t>
+          <t>Gap Detection Module - Classification Logic &amp; Test Report</t>
         </is>
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>Commitment extraction precision/recall targets (&gt;=85%/&gt;=90%) require validation against representative financial services email samples. Privacy-by-design constraints limit training data options.</t>
+          <t>Gap detection recall target &gt;=95% requires validation against representative client governance data. False positive rate must stay &lt;=10% to maintain PMO trust.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>1.3.2</t>
+          <t>1.3.3</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Cross-Source Task Consolidation &amp; Deduplication</t>
+          <t>Governance Scorecard Generator</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Build the consolidation layer merging tasks from email extraction, Wave 1 meeting action items, and JIRA assigned tickets into a single deduplicated list within the EPAM platform. Links related items across sources (e.g. email commitment matched to open JIRA ticket).</t>
+          <t>Develop per-project and portfolio-level governance scorecard views within the EPAM platform. Each project scorecard shows status (Compliant, At Risk, Non-Compliant) for every applicable standard, plus trend versus the previous assessment. Portfolio view shows governance health across all active projects. Scorecards are producible on demand for steering committee or audit use. Presented as drafts for PMO review - not distributed automatically.</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+          <t>Wave 2 Governance Monitoring delivers continuous automated assessment of every active project against configured governance standards - checking documentation, approvals, and gate criteria. It draws on Wave 1 RAID logs and decision records as primary evidence, generates per-project governance scorecards, detects gaps by type and severity, and surfaces escalation drafts for PMO review. All gap resolutions require explicit PMO action - the system detects and surfaces, humans resolve and dismiss.</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -1740,12 +1820,12 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F37" s="21" t="n">
+      <c r="F37" s="52" t="n">
         <v>46488</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Consolidation Engine - Deduplication Logic &amp; Test Report</t>
+          <t>Scorecard Generator - UX Spec &amp; Acceptance Criteria</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -1757,22 +1837,22 @@
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>1.3.3</t>
+          <t>1.3.4</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Prioritisation Engine &amp; Completion Detection</t>
+          <t>Escalation Notification &amp; Resolution Workflow (EPAM Web App)</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Build multi-factor prioritisation ranking tasks by due date, requester seniority, project priority, and RAID context. Implement completion detection via Outlook sent folder monitoring (Graph API) and JIRA status change tracking. Auto-close completed tasks in EPAM platform where evidence is clear; flag uncertain cases for PMO confirmation.</t>
+          <t>Build the governance alert and resolution interface in the EPAM React web application: weekly governance summary via Teams/Outlook, immediate High severity gap notifications with deep links into the platform, and a resolution workflow (Resolved, In Progress, Escalated, or Dismissed - dismissal requires a mandatory reason). Draft escalation notices for High severity gaps presented for PMO review and Outlook send. Full audit trail stored in Azure Table Storage.</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+          <t>Wave 2 Governance Monitoring delivers continuous automated assessment of every active project against configured governance standards - checking documentation, approvals, and gate criteria. It draws on Wave 1 RAID logs and decision records as primary evidence, generates per-project governance scorecards, detects gaps by type and severity, and surfaces escalation drafts for PMO review. All gap resolutions require explicit PMO action - the system detects and surfaces, humans resolve and dismiss.</t>
         </is>
       </c>
       <c r="E38" s="20" t="inlineStr">
@@ -1780,128 +1860,168 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F38" s="21" t="n">
+      <c r="F38" s="52" t="n">
+        <v>46516</v>
+      </c>
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>Governance Interface - UX Spec &amp; UAT Report</t>
+        </is>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>None at this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>1.4  Wave 2c - Stakeholder Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Deliverable Name</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Deliverable Description</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Project Description</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Delivery Owner</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Document Name</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Technological Uncertainties</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>1.4.1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Trigger Detection &amp; Context Gathering Agent</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Build the agent continuously monitoring the EPAM platform for trigger events: RAG status deterioration, milestone slip, new High severity Risk or Issue (from Wave 1), governance gap escalation (from Wave 2b Governance Monitoring), and milestone completion. For each trigger, the agent automatically gathers project context from Wave 1 RAID items and decisions, Wave 2 status report and RAG history, governance gap records, and JIRA ticket status. Trigger rules are configurable per client.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Wave 2 Stakeholder Communications delivers event-driven, context-aware draft communications triggered automatically by project events. It draws on Wave 1 meeting intelligence, Wave 2 status report data, and governance monitoring outputs to generate accurate audience-adapted drafts. All drafts require PMO review and approval - the AI never sends independently.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F41" s="55" t="n">
+        <v>46459</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Trigger Detection Agent - Logic Spec &amp; Test Report</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Trigger detection accuracy target &gt;=95% with &lt;=10% false trigger rate must be validated against representative client data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>1.4.2</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>Communication Draft Generation Agent</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>Develop the LLM-based agent generating draft communications from gathered context, covering: escalation notices (RAG change), milestone slip notifications, risk/issue escalations to sponsor, governance gap notices, milestone completion announcements, and steering committee briefings. Every factual statement must be traceable to a named source (RAID log, status data, JIRA ticket, or meeting decision). Confidence scoring flags low-confidence elements for extra PMO attention.</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>Wave 2 Stakeholder Communications delivers event-driven, context-aware draft communications triggered automatically by project events. It draws on Wave 1 meeting intelligence, Wave 2 status report data, and governance monitoring outputs to generate accurate, audience-adapted drafts for escalation notices, steering committee briefings, risk escalations, and milestone communications. All drafts are presented within the EPAM platform for PMO review and approval - the AI never sends independently.</t>
+        </is>
+      </c>
+      <c r="E42" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F42" s="52" t="n">
         <v>46488</v>
       </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>Prioritisation &amp; Detection - Logic Spec &amp; Test Report</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>None at this time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="18" t="inlineStr">
-        <is>
-          <t>1.3.4</t>
-        </is>
-      </c>
-      <c r="B39" s="18" t="inlineStr">
-        <is>
-          <t>Reminder Engine &amp; Daily Checklist Interface (EPAM Web App)</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>Develop reminder generation and delivery via Microsoft Graph API (Teams messages and Outlook emails), directing PMOs into the EPAM platform to take action. Build the daily checklist screen within the EPAM React web application - prioritised task list with manual tick-off, completion rate tracking, and mobile-responsive layout. Accessible via browser, no client-side installation required.</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
-        </is>
-      </c>
-      <c r="E39" s="20" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F39" s="21" t="n">
-        <v>46516</v>
-      </c>
-      <c r="G39" s="19" t="inlineStr">
-        <is>
-          <t>Checklist Interface - UX Spec &amp; UAT Report</t>
-        </is>
-      </c>
-      <c r="H39" s="19" t="inlineStr">
-        <is>
-          <t>None at this time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>1.4  Wave 2c - Strategic Resourcing</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="14" customHeight="1">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="inlineStr">
-        <is>
-          <t>Deliverable Name</t>
-        </is>
-      </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>Deliverable Description</t>
-        </is>
-      </c>
-      <c r="D42" s="17" t="inlineStr">
-        <is>
-          <t>Project Description</t>
-        </is>
-      </c>
-      <c r="E42" s="17" t="inlineStr">
-        <is>
-          <t>Delivery Owner</t>
-        </is>
-      </c>
-      <c r="F42" s="17" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>Document Name</t>
-        </is>
-      </c>
-      <c r="H42" s="17" t="inlineStr">
-        <is>
-          <t>Technological Uncertainties</t>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>Draft Generation Agent - Evaluation Report &amp; Source Traceability Spec</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>Draft acceptance rate target &gt;=75% (PMO sends without material changes) requires LLM prompt tuning and evaluation against representative financial services communications.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.3</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Resource Tracking &amp; Gap Detection Agent</t>
+          <t>Audience Adaptation &amp; Template Engine</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Build continuous monitoring agent reading resource end dates from client SharePoint/MS Project via Microsoft Graph API. Detects upcoming gaps within configurable lead time (default 4-6 weeks), cross-references against confirmed project demand, and surfaces prioritised gap alerts with confidence levels within the EPAM platform.</t>
+          <t>Build the audience adaptation layer generating separate, appropriately toned draft versions for different recipient types (sponsor, programme director, project team, executive, steering committee) from the same underlying context. Configurable communication templates and tone guidelines per client - PMO Lead can update without code changes. Duplicate draft suppression prevents re-generation for the same trigger event while a draft is pending review.</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Strategic Resourcing makes resource management proactive. The EPAM platform continuously monitors project end dates by reading from client SharePoint resource trackers and MS Project via API, detects upcoming gaps before they occur, maintains a queryable skills inventory, and recommends best-fit resource matches with explicit trade-off reasoning. Resource gap alerts and match recommendations are surfaced within the EPAM browser-based platform. Resource commitments are always human-confirmed - the AI informs the decision, never makes it.</t>
+          <t>Wave 2 Stakeholder Communications delivers event-driven, context-aware draft communications triggered automatically by project events. It draws on Wave 1 meeting intelligence, Wave 2 status report data, and governance monitoring outputs to generate accurate, audience-adapted drafts for escalation notices, steering committee briefings, risk escalations, and milestone communications. All drafts are presented within the EPAM platform for PMO review and approval - the AI never sends independently.</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -1909,135 +2029,474 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="F43" s="21" t="n">
+      <c r="F43" s="52" t="n">
         <v>46488</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Resource Tracking Agent - Alert Logic &amp; Test Report</t>
+          <t>Audience Adaptation Engine - Template Spec &amp; Config Guide</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>Data quality in client resource trackers is variable. A data quality assessment and potential remediation phase may be required before reliable gap detection is achievable.</t>
+          <t>None at this time.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>1.4.4</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
+          <t>Review, Approval &amp; Outlook Distribution Workflow (EPAM Web App)</t>
+        </is>
+      </c>
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>Build the communication review and approval screen within the EPAM React web application: draft presentation with inline editing (subject, recipient, body text), approve-and-send via Outlook (Microsoft Graph API), discard without reason required, and pending-review reminders via Teams/Outlook for drafts unreviewed beyond a configurable period. Approved communications logged with original draft, PMO edits, approving user, timestamp, and recipient list. Optional write-back to SharePoint project records where configured.</t>
+        </is>
+      </c>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>Wave 2 Stakeholder Communications delivers event-driven, context-aware draft communications triggered automatically by project events. It draws on Wave 1 meeting intelligence, Wave 2 status report data, and governance monitoring outputs to generate accurate, audience-adapted drafts for escalation notices, steering committee briefings, risk escalations, and milestone communications. All drafts are presented within the EPAM platform for PMO review and approval - the AI never sends independently.</t>
+        </is>
+      </c>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F44" s="52" t="n">
+        <v>46516</v>
+      </c>
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>Comms Interface - UX Spec &amp; UAT Report</t>
+        </is>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
+        <is>
+          <t>None at this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1"/>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>1.5  Wave 3a - Personal Task Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Deliverable Name</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Deliverable Description</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Project Description</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Delivery Owner</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>Document Name</t>
+        </is>
+      </c>
+      <c r="H47" s="17" t="inlineStr">
+        <is>
+          <t>Technological Uncertainties</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>1.5.1</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t>Email Commitment Extraction Agent</t>
+        </is>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>Develop the LLM-based agent that connects to the PMO Outlook inbox via Microsoft Graph API, scans over a configurable lookback window (default 3 days), identifies commitments made by and tasks directed at the PMO, and distinguishes hard commitments from soft commitments and FYI information. Extracted tasks surfaced in the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F48" s="52" t="n">
+        <v>46459</v>
+      </c>
+      <c r="G48" s="19" t="inlineStr">
+        <is>
+          <t>Email Agent - Accuracy Evaluation &amp; PII Handling Report</t>
+        </is>
+      </c>
+      <c r="H48" s="19" t="inlineStr">
+        <is>
+          <t>Commitment extraction precision/recall targets (&gt;=85%/&gt;=90%) require validation against representative financial services email samples. Privacy-by-design constraints limit training data options.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>1.5.2</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Cross-Source Task Consolidation &amp; Deduplication</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>Build the consolidation layer merging tasks from email extraction, Wave 1 meeting action items, and JIRA assigned tickets into a single deduplicated list within the EPAM platform. Links related items across sources (e.g. email commitment matched to open JIRA ticket).</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F49" s="52" t="n">
+        <v>46488</v>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Consolidation Engine - Deduplication Logic &amp; Test Report</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>None at this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>1.5.3</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>Prioritisation Engine &amp; Completion Detection</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>Build multi-factor prioritisation ranking tasks by due date, requester seniority, project priority, and RAID context. Implement completion detection via Outlook sent folder monitoring (Graph API) and JIRA status change tracking. Auto-close completed tasks in EPAM platform where evidence is clear; flag uncertain cases for PMO confirmation.</t>
+        </is>
+      </c>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F50" s="52" t="n">
+        <v>46488</v>
+      </c>
+      <c r="G50" s="19" t="inlineStr">
+        <is>
+          <t>Prioritisation &amp; Detection - Logic Spec &amp; Test Report</t>
+        </is>
+      </c>
+      <c r="H50" s="19" t="inlineStr">
+        <is>
+          <t>None at this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
+        <is>
+          <t>1.5.4</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>Reminder Engine &amp; Daily Checklist Interface (EPAM Web App)</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Develop reminder generation and delivery via Microsoft Graph API (Teams messages and Outlook emails), directing PMOs into the EPAM platform to take action. Build the daily checklist screen within the EPAM React web application - prioritised task list with manual tick-off, completion rate tracking, and mobile-responsive layout. Accessible via browser, no client-side installation required.</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Personal Task Management consolidates all PMO commitments - extracted from Outlook email, Wave 1 meeting action items, and JIRA - into a single prioritised daily task list presented within the EPAM web platform. The system automatically detects completions, generates contextual reminders delivered via Teams or Outlook, and provides a clean browser-based daily checklist interface. No task management tooling is installed on client machines - everything runs through the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F51" s="52" t="n">
+        <v>46516</v>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>Checklist Interface - UX Spec &amp; UAT Report</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>None at this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>1.6  Wave 3b - Strategic Resourcing</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Deliverable Name</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>Deliverable Description</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Project Description</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Delivery Owner</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>Document Name</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="inlineStr">
+        <is>
+          <t>Technological Uncertainties</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>Resource Tracking &amp; Gap Detection Agent</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Build continuous monitoring agent reading resource end dates from client SharePoint/MS Project via Microsoft Graph API. Detects upcoming gaps within configurable lead time (default 4-6 weeks), cross-references against confirmed project demand, and surfaces prioritised gap alerts with confidence levels within the EPAM platform.</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Strategic Resourcing makes resource management proactive. The EPAM platform continuously monitors project end dates by reading from client SharePoint resource trackers and MS Project via API, detects upcoming gaps before they occur, maintains a queryable skills inventory, and recommends best-fit resource matches with explicit trade-off reasoning. Resource gap alerts and match recommendations are surfaced within the EPAM browser-based platform. Resource commitments are always human-confirmed - the AI informs the decision, never makes it.</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F55" s="52" t="n">
+        <v>46488</v>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
+          <t>Resource Tracking Agent - Alert Logic &amp; Test Report</t>
+        </is>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>Data quality in client resource trackers is variable. A data quality assessment and potential remediation phase may be required before reliable gap detection is achievable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>1.6.2</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
           <t>Skills Inventory Management</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C56" s="19" t="inlineStr">
         <is>
           <t>Build queryable skills and experience database within the EPAM platform with configurable taxonomy per client. Implement staleness detection (default 90-day refresh prompt). PMO update interface within the EPAM web app with full change audit log. Integration with HR system API where available.</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
+      <c r="D56" s="19" t="inlineStr">
         <is>
           <t>Strategic Resourcing makes resource management proactive. The EPAM platform continuously monitors project end dates by reading from client SharePoint resource trackers and MS Project via API, detects upcoming gaps before they occur, maintains a queryable skills inventory, and recommends best-fit resource matches with explicit trade-off reasoning. Resource gap alerts and match recommendations are surfaced within the EPAM browser-based platform. Resource commitments are always human-confirmed - the AI informs the decision, never makes it.</t>
         </is>
       </c>
-      <c r="E44" s="20" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F44" s="21" t="n">
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F56" s="52" t="n">
         <v>46488</v>
       </c>
-      <c r="G44" s="19" t="inlineStr">
+      <c r="G56" s="19" t="inlineStr">
         <is>
           <t>Skills Inventory - Schema Design &amp; Config Spec</t>
         </is>
       </c>
-      <c r="H44" s="19" t="inlineStr">
+      <c r="H56" s="19" t="inlineStr">
         <is>
           <t>HR system API availability varies by client. Where no API exists, skills data must be seeded and maintained manually via the EPAM platform UI.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="60" customHeight="1">
-      <c r="A45" s="18" t="inlineStr">
-        <is>
-          <t>1.4.3</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="18" t="inlineStr">
+        <is>
+          <t>1.6.3</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
         <is>
           <t>Match Recommendation Engine</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>Develop multi-factor matching algorithm recommending best-fit resources for identified gaps, weighing: availability, skill match, seniority, sector experience, and project priority. Presents ranked candidates with explicit trade-off explanations within the EPAM platform. Flags where no internal fit exists.</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>Strategic Resourcing makes resource management proactive. The EPAM platform continuously monitors project end dates by reading from client SharePoint resource trackers and MS Project via API, detects upcoming gaps before they occur, maintains a queryable skills inventory, and recommends best-fit resource matches with explicit trade-off reasoning. Resource gap alerts and match recommendations are surfaced within the EPAM browser-based platform. Resource commitments are always human-confirmed - the AI informs the decision, never makes it.</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F45" s="21" t="n">
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F57" s="52" t="n">
         <v>46516</v>
       </c>
-      <c r="G45" s="19" t="inlineStr">
+      <c r="G57" s="19" t="inlineStr">
         <is>
           <t>Match Engine - Algorithm Spec &amp; Acceptance Criteria</t>
         </is>
       </c>
-      <c r="H45" s="19" t="inlineStr">
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>Recommendation quality degrades with incomplete skills inventory data. Minimum viable inventory coverage (&gt;=90%) is a prerequisite for reliable matching.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1">
-      <c r="A46" s="18" t="inlineStr">
-        <is>
-          <t>1.4.4</t>
-        </is>
-      </c>
-      <c r="B46" s="18" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>1.6.4</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
         <is>
           <t>Resource Alert Interface &amp; Approval Workflow (EPAM Web App)</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>Build the resource alert and approval screen within the EPAM React web application: gap alert detail, ranked match recommendations with trade-off explanations, and resource assignment confirmation. Enforce human-only resource commitment at the workflow level. Confirmed assignments automatically update client resource tracker and project record via API.</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>Strategic Resourcing makes resource management proactive. The EPAM platform continuously monitors project end dates by reading from client SharePoint resource trackers and MS Project via API, detects upcoming gaps before they occur, maintains a queryable skills inventory, and recommends best-fit resource matches with explicit trade-off reasoning. Resource gap alerts and match recommendations are surfaced within the EPAM browser-based platform. Resource commitments are always human-confirmed - the AI informs the decision, never makes it.</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F46" s="21" t="n">
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F58" s="52" t="n">
         <v>46516</v>
       </c>
-      <c r="G46" s="19" t="inlineStr">
+      <c r="G58" s="19" t="inlineStr">
         <is>
           <t>Resourcing Interface - UX Spec &amp; Governance Workflow</t>
         </is>
       </c>
-      <c r="H46" s="19" t="inlineStr">
+      <c r="H58" s="19" t="inlineStr">
         <is>
           <t>None at this time.</t>
         </is>
@@ -2046,11 +2505,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2062,7 +2521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T34"/>
+  <dimension ref="A1:T42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3097,54 +3556,54 @@
       <c r="T20" s="34" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>1.3.1</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
-        <is>
-          <t>Personal Tasks</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>Email Commitment Extraction Agent</t>
-        </is>
-      </c>
-      <c r="D21" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E21" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>Governance Monitoring</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>Governance Standards Config &amp; Assessment Engine</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G21" s="27" t="n"/>
-      <c r="H21" s="25" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="I21" s="29" t="inlineStr"/>
-      <c r="J21" s="29" t="inlineStr"/>
-      <c r="K21" s="29" t="inlineStr"/>
-      <c r="L21" s="29" t="inlineStr"/>
-      <c r="M21" s="29" t="inlineStr"/>
-      <c r="N21" s="37" t="inlineStr"/>
-      <c r="O21" s="37" t="inlineStr"/>
-      <c r="P21" s="29" t="inlineStr"/>
-      <c r="Q21" s="29" t="inlineStr"/>
-      <c r="R21" s="29" t="inlineStr"/>
-      <c r="S21" s="29" t="inlineStr"/>
-      <c r="T21" s="29" t="inlineStr"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I21" s="34" t="n"/>
+      <c r="J21" s="34" t="n"/>
+      <c r="K21" s="34" t="n"/>
+      <c r="L21" s="34" t="n"/>
+      <c r="M21" s="34" t="n"/>
+      <c r="N21" s="37" t="n"/>
+      <c r="O21" s="37" t="n"/>
+      <c r="P21" s="34" t="n"/>
+      <c r="Q21" s="34" t="n"/>
+      <c r="R21" s="34" t="n"/>
+      <c r="S21" s="34" t="n"/>
+      <c r="T21" s="34" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="30" t="inlineStr">
@@ -3154,12 +3613,12 @@
       </c>
       <c r="B22" s="31" t="inlineStr">
         <is>
-          <t>Personal Tasks</t>
+          <t>Governance Monitoring</t>
         </is>
       </c>
       <c r="C22" s="32" t="inlineStr">
         <is>
-          <t>Cross-Source Consolidation</t>
+          <t>Gap Detection &amp; Classification Module</t>
         </is>
       </c>
       <c r="D22" s="33" t="inlineStr">
@@ -3183,68 +3642,68 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="I22" s="34" t="inlineStr"/>
-      <c r="J22" s="34" t="inlineStr"/>
-      <c r="K22" s="34" t="inlineStr"/>
-      <c r="L22" s="34" t="inlineStr"/>
-      <c r="M22" s="34" t="inlineStr"/>
-      <c r="N22" s="34" t="inlineStr"/>
-      <c r="O22" s="37" t="inlineStr"/>
-      <c r="P22" s="37" t="inlineStr"/>
-      <c r="Q22" s="34" t="inlineStr"/>
-      <c r="R22" s="34" t="inlineStr"/>
-      <c r="S22" s="34" t="inlineStr"/>
-      <c r="T22" s="34" t="inlineStr"/>
+      <c r="I22" s="34" t="n"/>
+      <c r="J22" s="34" t="n"/>
+      <c r="K22" s="34" t="n"/>
+      <c r="L22" s="34" t="n"/>
+      <c r="M22" s="34" t="n"/>
+      <c r="N22" s="37" t="n"/>
+      <c r="O22" s="37" t="n"/>
+      <c r="P22" s="34" t="n"/>
+      <c r="Q22" s="34" t="n"/>
+      <c r="R22" s="34" t="n"/>
+      <c r="S22" s="34" t="n"/>
+      <c r="T22" s="34" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>1.3.3</t>
         </is>
       </c>
-      <c r="B23" s="25" t="inlineStr">
-        <is>
-          <t>Personal Tasks</t>
-        </is>
-      </c>
-      <c r="C23" s="26" t="inlineStr">
-        <is>
-          <t>Prioritisation &amp; Completion Detection</t>
-        </is>
-      </c>
-      <c r="D23" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E23" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>Governance Monitoring</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Governance Scorecard Generator</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G23" s="27" t="n"/>
-      <c r="H23" s="25" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="I23" s="29" t="inlineStr"/>
-      <c r="J23" s="29" t="inlineStr"/>
-      <c r="K23" s="29" t="inlineStr"/>
-      <c r="L23" s="29" t="inlineStr"/>
-      <c r="M23" s="29" t="inlineStr"/>
-      <c r="N23" s="29" t="inlineStr"/>
-      <c r="O23" s="37" t="inlineStr"/>
-      <c r="P23" s="37" t="inlineStr"/>
-      <c r="Q23" s="29" t="inlineStr"/>
-      <c r="R23" s="29" t="inlineStr"/>
-      <c r="S23" s="29" t="inlineStr"/>
-      <c r="T23" s="29" t="inlineStr"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I23" s="34" t="n"/>
+      <c r="J23" s="34" t="n"/>
+      <c r="K23" s="34" t="n"/>
+      <c r="L23" s="34" t="n"/>
+      <c r="M23" s="34" t="n"/>
+      <c r="N23" s="37" t="n"/>
+      <c r="O23" s="37" t="n"/>
+      <c r="P23" s="34" t="n"/>
+      <c r="Q23" s="34" t="n"/>
+      <c r="R23" s="34" t="n"/>
+      <c r="S23" s="34" t="n"/>
+      <c r="T23" s="34" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="30" t="inlineStr">
@@ -3254,12 +3713,12 @@
       </c>
       <c r="B24" s="31" t="inlineStr">
         <is>
-          <t>Personal Tasks</t>
+          <t>Governance Monitoring</t>
         </is>
       </c>
       <c r="C24" s="32" t="inlineStr">
         <is>
-          <t>Reminder Engine &amp; Checklist Interface</t>
+          <t>Escalation Notification &amp; Resolution Workflow</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
@@ -3283,68 +3742,68 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="I24" s="34" t="inlineStr"/>
-      <c r="J24" s="34" t="inlineStr"/>
-      <c r="K24" s="34" t="inlineStr"/>
-      <c r="L24" s="34" t="inlineStr"/>
-      <c r="M24" s="34" t="inlineStr"/>
-      <c r="N24" s="34" t="inlineStr"/>
-      <c r="O24" s="34" t="inlineStr"/>
-      <c r="P24" s="37" t="inlineStr"/>
-      <c r="Q24" s="37" t="inlineStr"/>
-      <c r="R24" s="34" t="inlineStr"/>
-      <c r="S24" s="34" t="inlineStr"/>
-      <c r="T24" s="34" t="inlineStr"/>
+      <c r="I24" s="34" t="n"/>
+      <c r="J24" s="34" t="n"/>
+      <c r="K24" s="34" t="n"/>
+      <c r="L24" s="34" t="n"/>
+      <c r="M24" s="34" t="n"/>
+      <c r="N24" s="37" t="n"/>
+      <c r="O24" s="37" t="n"/>
+      <c r="P24" s="34" t="n"/>
+      <c r="Q24" s="34" t="n"/>
+      <c r="R24" s="34" t="n"/>
+      <c r="S24" s="34" t="n"/>
+      <c r="T24" s="34" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>1.4.1</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>Strategic Resourcing</t>
-        </is>
-      </c>
-      <c r="C25" s="26" t="inlineStr">
-        <is>
-          <t>Resource Tracking &amp; Gap Detection</t>
-        </is>
-      </c>
-      <c r="D25" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E25" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>Stakeholder Communications</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>Trigger Detection &amp; Context Gathering Agent</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G25" s="27" t="n"/>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="I25" s="29" t="inlineStr"/>
-      <c r="J25" s="29" t="inlineStr"/>
-      <c r="K25" s="29" t="inlineStr"/>
-      <c r="L25" s="29" t="inlineStr"/>
-      <c r="M25" s="29" t="inlineStr"/>
-      <c r="N25" s="29" t="inlineStr"/>
-      <c r="O25" s="37" t="inlineStr"/>
-      <c r="P25" s="37" t="inlineStr"/>
-      <c r="Q25" s="29" t="inlineStr"/>
-      <c r="R25" s="29" t="inlineStr"/>
-      <c r="S25" s="29" t="inlineStr"/>
-      <c r="T25" s="29" t="inlineStr"/>
+      <c r="G25" s="33" t="n"/>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I25" s="34" t="n"/>
+      <c r="J25" s="34" t="n"/>
+      <c r="K25" s="34" t="n"/>
+      <c r="L25" s="34" t="n"/>
+      <c r="M25" s="34" t="n"/>
+      <c r="N25" s="37" t="n"/>
+      <c r="O25" s="37" t="n"/>
+      <c r="P25" s="34" t="n"/>
+      <c r="Q25" s="34" t="n"/>
+      <c r="R25" s="34" t="n"/>
+      <c r="S25" s="34" t="n"/>
+      <c r="T25" s="34" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="30" t="inlineStr">
@@ -3354,12 +3813,12 @@
       </c>
       <c r="B26" s="31" t="inlineStr">
         <is>
-          <t>Strategic Resourcing</t>
+          <t>Stakeholder Communications</t>
         </is>
       </c>
       <c r="C26" s="32" t="inlineStr">
         <is>
-          <t>Skills Inventory Management</t>
+          <t>Communication Draft Generation Agent</t>
         </is>
       </c>
       <c r="D26" s="33" t="inlineStr">
@@ -3383,68 +3842,68 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="I26" s="34" t="inlineStr"/>
-      <c r="J26" s="34" t="inlineStr"/>
-      <c r="K26" s="34" t="inlineStr"/>
-      <c r="L26" s="34" t="inlineStr"/>
-      <c r="M26" s="34" t="inlineStr"/>
-      <c r="N26" s="34" t="inlineStr"/>
-      <c r="O26" s="37" t="inlineStr"/>
-      <c r="P26" s="37" t="inlineStr"/>
-      <c r="Q26" s="34" t="inlineStr"/>
-      <c r="R26" s="34" t="inlineStr"/>
-      <c r="S26" s="34" t="inlineStr"/>
-      <c r="T26" s="34" t="inlineStr"/>
+      <c r="I26" s="34" t="n"/>
+      <c r="J26" s="34" t="n"/>
+      <c r="K26" s="34" t="n"/>
+      <c r="L26" s="34" t="n"/>
+      <c r="M26" s="34" t="n"/>
+      <c r="N26" s="37" t="n"/>
+      <c r="O26" s="37" t="n"/>
+      <c r="P26" s="34" t="n"/>
+      <c r="Q26" s="34" t="n"/>
+      <c r="R26" s="34" t="n"/>
+      <c r="S26" s="34" t="n"/>
+      <c r="T26" s="34" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="24" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>1.4.3</t>
         </is>
       </c>
-      <c r="B27" s="25" t="inlineStr">
-        <is>
-          <t>Strategic Resourcing</t>
-        </is>
-      </c>
-      <c r="C27" s="26" t="inlineStr">
-        <is>
-          <t>Match Recommendation Engine</t>
-        </is>
-      </c>
-      <c r="D27" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="E27" s="27" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>Stakeholder Communications</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>Audience Adaptation &amp; Template Engine</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G27" s="27" t="n"/>
-      <c r="H27" s="25" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="I27" s="29" t="inlineStr"/>
-      <c r="J27" s="29" t="inlineStr"/>
-      <c r="K27" s="29" t="inlineStr"/>
-      <c r="L27" s="29" t="inlineStr"/>
-      <c r="M27" s="29" t="inlineStr"/>
-      <c r="N27" s="29" t="inlineStr"/>
-      <c r="O27" s="29" t="inlineStr"/>
-      <c r="P27" s="37" t="inlineStr"/>
-      <c r="Q27" s="37" t="inlineStr"/>
-      <c r="R27" s="29" t="inlineStr"/>
-      <c r="S27" s="29" t="inlineStr"/>
-      <c r="T27" s="29" t="inlineStr"/>
+      <c r="G27" s="33" t="n"/>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I27" s="34" t="n"/>
+      <c r="J27" s="34" t="n"/>
+      <c r="K27" s="34" t="n"/>
+      <c r="L27" s="34" t="n"/>
+      <c r="M27" s="34" t="n"/>
+      <c r="N27" s="37" t="n"/>
+      <c r="O27" s="37" t="n"/>
+      <c r="P27" s="34" t="n"/>
+      <c r="Q27" s="34" t="n"/>
+      <c r="R27" s="34" t="n"/>
+      <c r="S27" s="34" t="n"/>
+      <c r="T27" s="34" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="30" t="inlineStr">
@@ -3454,12 +3913,12 @@
       </c>
       <c r="B28" s="31" t="inlineStr">
         <is>
-          <t>Strategic Resourcing</t>
+          <t>Stakeholder Communications</t>
         </is>
       </c>
       <c r="C28" s="32" t="inlineStr">
         <is>
-          <t>Resource Alert Interface (EPAM Web App)</t>
+          <t>Review, Approval &amp; Outlook Distribution Workflow</t>
         </is>
       </c>
       <c r="D28" s="33" t="inlineStr">
@@ -3483,53 +3942,381 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="I28" s="34" t="inlineStr"/>
-      <c r="J28" s="34" t="inlineStr"/>
-      <c r="K28" s="34" t="inlineStr"/>
-      <c r="L28" s="34" t="inlineStr"/>
-      <c r="M28" s="34" t="inlineStr"/>
-      <c r="N28" s="34" t="inlineStr"/>
-      <c r="O28" s="34" t="inlineStr"/>
-      <c r="P28" s="37" t="inlineStr"/>
-      <c r="Q28" s="37" t="inlineStr"/>
-      <c r="R28" s="34" t="inlineStr"/>
-      <c r="S28" s="34" t="inlineStr"/>
-      <c r="T28" s="34" t="inlineStr"/>
+      <c r="I28" s="34" t="n"/>
+      <c r="J28" s="34" t="n"/>
+      <c r="K28" s="34" t="n"/>
+      <c r="L28" s="34" t="n"/>
+      <c r="M28" s="34" t="n"/>
+      <c r="N28" s="37" t="n"/>
+      <c r="O28" s="37" t="n"/>
+      <c r="P28" s="34" t="n"/>
+      <c r="Q28" s="34" t="n"/>
+      <c r="R28" s="34" t="n"/>
+      <c r="S28" s="34" t="n"/>
+      <c r="T28" s="34" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>1.5.1</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="inlineStr">
+        <is>
+          <t>Personal Tasks (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Email Commitment Extraction Agent</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G29" s="27" t="n"/>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I29" s="29" t="inlineStr"/>
+      <c r="J29" s="29" t="inlineStr"/>
+      <c r="K29" s="29" t="inlineStr"/>
+      <c r="L29" s="29" t="inlineStr"/>
+      <c r="M29" s="29" t="inlineStr"/>
+      <c r="N29" s="37" t="inlineStr"/>
+      <c r="O29" s="37" t="inlineStr"/>
+      <c r="P29" s="29" t="inlineStr"/>
+      <c r="Q29" s="29" t="inlineStr"/>
+      <c r="R29" s="29" t="inlineStr"/>
+      <c r="S29" s="29" t="inlineStr"/>
+      <c r="T29" s="29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>1.5.2</t>
+        </is>
+      </c>
+      <c r="B30" s="53" t="n"/>
+      <c r="C30" s="54" t="n"/>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F30" s="33" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I30" s="34" t="inlineStr"/>
+      <c r="J30" s="34" t="inlineStr"/>
+      <c r="K30" s="34" t="inlineStr"/>
+      <c r="L30" s="34" t="inlineStr"/>
+      <c r="M30" s="34" t="inlineStr"/>
+      <c r="N30" s="34" t="inlineStr"/>
+      <c r="O30" s="37" t="inlineStr"/>
+      <c r="P30" s="37" t="inlineStr"/>
+      <c r="Q30" s="34" t="inlineStr"/>
+      <c r="R30" s="34" t="inlineStr"/>
+      <c r="S30" s="34" t="inlineStr"/>
+      <c r="T30" s="34" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>1.5.3</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="inlineStr">
+        <is>
+          <t>Personal Tasks (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C31" s="53" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="54" t="n"/>
+      <c r="G31" s="27" t="n"/>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I31" s="29" t="inlineStr"/>
+      <c r="J31" s="29" t="inlineStr"/>
+      <c r="K31" s="29" t="inlineStr"/>
+      <c r="L31" s="29" t="inlineStr"/>
+      <c r="M31" s="29" t="inlineStr"/>
+      <c r="N31" s="29" t="inlineStr"/>
+      <c r="O31" s="37" t="inlineStr"/>
+      <c r="P31" s="37" t="inlineStr"/>
+      <c r="Q31" s="29" t="inlineStr"/>
+      <c r="R31" s="29" t="inlineStr"/>
+      <c r="S31" s="29" t="inlineStr"/>
+      <c r="T31" s="29" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>1.5.4</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Personal Tasks (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="53" t="n"/>
+      <c r="F32" s="54" t="n"/>
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I32" s="34" t="inlineStr"/>
+      <c r="J32" s="34" t="inlineStr"/>
+      <c r="K32" s="34" t="inlineStr"/>
+      <c r="L32" s="34" t="inlineStr"/>
+      <c r="M32" s="34" t="inlineStr"/>
+      <c r="N32" s="34" t="inlineStr"/>
+      <c r="O32" s="34" t="inlineStr"/>
+      <c r="P32" s="37" t="inlineStr"/>
+      <c r="Q32" s="37" t="inlineStr"/>
+      <c r="R32" s="34" t="inlineStr"/>
+      <c r="S32" s="34" t="inlineStr"/>
+      <c r="T32" s="34" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>1.6.1</t>
+        </is>
+      </c>
+      <c r="B33" s="25" t="inlineStr">
+        <is>
+          <t>Strategic Resourcing (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C33" s="53" t="n"/>
+      <c r="D33" s="53" t="n"/>
+      <c r="E33" s="53" t="n"/>
+      <c r="F33" s="54" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I33" s="29" t="inlineStr"/>
+      <c r="J33" s="29" t="inlineStr"/>
+      <c r="K33" s="29" t="inlineStr"/>
+      <c r="L33" s="29" t="inlineStr"/>
+      <c r="M33" s="29" t="inlineStr"/>
+      <c r="N33" s="29" t="inlineStr"/>
+      <c r="O33" s="37" t="inlineStr"/>
+      <c r="P33" s="37" t="inlineStr"/>
+      <c r="Q33" s="29" t="inlineStr"/>
+      <c r="R33" s="29" t="inlineStr"/>
+      <c r="S33" s="29" t="inlineStr"/>
+      <c r="T33" s="29" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>1.6.2</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>Strategic Resourcing (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="n"/>
+      <c r="D34" s="53" t="n"/>
+      <c r="E34" s="53" t="n"/>
+      <c r="F34" s="54" t="n"/>
+      <c r="G34" s="33" t="n"/>
+      <c r="H34" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I34" s="34" t="inlineStr"/>
+      <c r="J34" s="34" t="inlineStr"/>
+      <c r="K34" s="34" t="inlineStr"/>
+      <c r="L34" s="34" t="inlineStr"/>
+      <c r="M34" s="34" t="inlineStr"/>
+      <c r="N34" s="34" t="inlineStr"/>
+      <c r="O34" s="37" t="inlineStr"/>
+      <c r="P34" s="37" t="inlineStr"/>
+      <c r="Q34" s="34" t="inlineStr"/>
+      <c r="R34" s="34" t="inlineStr"/>
+      <c r="S34" s="34" t="inlineStr"/>
+      <c r="T34" s="34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>1.6.3</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>Strategic Resourcing (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>Match Recommendation Engine</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G35" s="27" t="n"/>
+      <c r="H35" s="25" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I35" s="29" t="inlineStr"/>
+      <c r="J35" s="29" t="inlineStr"/>
+      <c r="K35" s="29" t="inlineStr"/>
+      <c r="L35" s="29" t="inlineStr"/>
+      <c r="M35" s="29" t="inlineStr"/>
+      <c r="N35" s="29" t="inlineStr"/>
+      <c r="O35" s="29" t="inlineStr"/>
+      <c r="P35" s="37" t="inlineStr"/>
+      <c r="Q35" s="37" t="inlineStr"/>
+      <c r="R35" s="29" t="inlineStr"/>
+      <c r="S35" s="29" t="inlineStr"/>
+      <c r="T35" s="29" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>1.6.4</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>Strategic Resourcing (Wave 3)</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>Resource Alert Interface (EPAM Web App)</t>
+        </is>
+      </c>
+      <c r="D36" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="E36" s="33" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="F36" s="33" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G36" s="33" t="n"/>
+      <c r="H36" s="31" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="I36" s="34" t="inlineStr"/>
+      <c r="J36" s="34" t="inlineStr"/>
+      <c r="K36" s="34" t="inlineStr"/>
+      <c r="L36" s="34" t="inlineStr"/>
+      <c r="M36" s="34" t="inlineStr"/>
+      <c r="N36" s="34" t="inlineStr"/>
+      <c r="O36" s="34" t="inlineStr"/>
+      <c r="P36" s="37" t="inlineStr"/>
+      <c r="Q36" s="37" t="inlineStr"/>
+      <c r="R36" s="34" t="inlineStr"/>
+      <c r="S36" s="34" t="inlineStr"/>
+      <c r="T36" s="34" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="39" t="n"/>
-      <c r="B31" s="40" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="39" t="n"/>
+      <c r="B39" s="40" t="inlineStr">
         <is>
           <t>Foundation - EPAM Platform Infrastructure (pre-Wave 1)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="41" t="n"/>
-      <c r="B32" s="40" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="41" t="n"/>
+      <c r="B40" s="40" t="inlineStr">
         <is>
           <t>Wave 1 - Meeting Intelligence</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="42" t="n"/>
-      <c r="B33" s="40" t="inlineStr">
-        <is>
-          <t>Wave 2 - Status Reports / Personal Tasks / Resourcing</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="40" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="42" t="n"/>
+      <c r="B41" s="40" t="inlineStr">
+        <is>
+          <t>Wave 2 - Status Reports / Governance Monitoring / Stakeholder Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="43" t="n"/>
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>Cross-cutting (runs across all waves)</t>
         </is>
@@ -3897,8 +4684,8 @@
           <t>Total Hours</t>
         </is>
       </c>
-      <c r="B42" s="47" t="n"/>
-      <c r="C42" s="47" t="n"/>
+      <c r="B42" s="53" t="n"/>
+      <c r="C42" s="54" t="n"/>
       <c r="D42" s="48">
         <f>SUM(D12:D41)</f>
         <v/>

</xml_diff>